<commit_message>
Atualização dos arquivos de metadados
</commit_message>
<xml_diff>
--- a/metadados/videos.xlsx
+++ b/metadados/videos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3968,6 +3968,216 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>como-manter-o-grind-diariamente.mp4</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>como-manter-a-determinacao-diariamente.mp4</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Como manter a determinação diariamente</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>É difícil manter o foco todos os dias? Descubra como se levantar e tentar novamente, mesmo quando está cansado. #DeterminacaoDiaria #CrescimentoPessoal</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>#DeterminacaoDiaria #CrescimentoPessoal #Persistencia</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>58</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2025-09-11 08:03:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>como-se-tornar-um-homem.mp4</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>por-que-voce-nao-tem-motivacao.mp4</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Por que você não tem motivação?</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Entenda o verdadeiro significado de disciplina e esforço contínuo. #Motivação #Disciplina</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>#Motivação #Disciplina #EsforçoContinuo</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>49</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2025-09-11 08:03:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>desabafando-sobre-motivacao.mp4</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>por-que-voce-nao-se-motiva.mp4</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Por que você não se motiva?</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Motivação, disciplina e persistência são as chaves para o sucesso. Descubra por que você pode estar parado e comece a agir agora! #motivação #disciplina #sucesso</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>#motivação #disciplina #sucesso</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>54</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2025-09-11 08:03:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>por-que-voce-nao-tem-amigos.mp4</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>por-que-voce-nao-esta-no-centro-das-atencoes.mp4</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Por que você não está no centro das atenções</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Aprenda a 'rub elbows' e conquiste seu espaço nos ambientes sociais. Por que esperar as pessoas te notarem quando você pode lutar por isso? #socialmedia #desenvolvimentopessoal</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>#rubelbows #sociais #atensao</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>56</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2025-09-11 08:03:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>por-que-voce-nao-vence.mp4</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>como-superar-a-falta-de-motivacao.mp4</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Como superar a falta de motivação</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Entenda por que a disciplina é fundamental para o sucesso. #Motivação #Disciplina #Sucesso</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>#Motivação #Disciplina #Sucesso</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>59</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2025-09-11 08:03:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>sobre-ser-um-underdog.mp4</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>por-que-voce-nao-vence-as-dificuldades.mp4</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Por que você não vence as dificuldades?</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Entenda as verdadeiras razões por trás de seus fracassos e comece a superar obstáculos com disciplina e determinação. #SuperandoDificuldades #Motivação</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>#SuperandoDificuldades #Motivação #Disciplina</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>59</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2025-09-11 08:03:59</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v8.0 - Dublagem com voz clonada funcionando
✅ FUNCIONALIDADES IMPLEMENTADAS:
- Download de vídeos perfeito
- Configuração completa (fonte, modo, qualidade, cor, posição)
- Cortes e legendas perfeitos
- Geração de textos AI (primeira etapa) funcionando
- Dublagem com voz clonada implementada
- Sincronização corrigida e funcionando
- GPU ativada e funcionando
- Correção PyTorch 2.6 weights_only
- Correção time-stretching (atempo inverso)

⚠️ MELHORIAS PENDENTES:
- Qualidade do timbre em partes rápidas
- Geração de textos AI para vídeos dublados
- Metadados específicos para vídeos dublados
- Renomeação automática de vídeos dublados

🎯 STATUS: Versão estável para desenvolvimento contínuo
</commit_message>
<xml_diff>
--- a/metadados/videos.xlsx
+++ b/metadados/videos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3968,6 +3968,426 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>corte_1_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>reconhecimento-de-padroes-para-sucesso.mp4</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Reconhecimento de padrões para sucesso</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Entenda por que Amazon é tão bem-sucedida e como Tom Brady utiliza padrões para o seu benefício. Aprenda a ver, usar e criar padrões no seu favor! #Padrão #Sucesso #TomBrady</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>#Padrão #Sucesso #TomBrady</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>40.03</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2025-09-12 20:59:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>corte_2_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>progresso-e-a-chave-para-a-felicidade.mp4</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Progresso é a chave para a felicidade</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Felicidade não vem de estatuetas ou riqueza, mas da constante evolução. #progresso #felicidade</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>#progresso #felicidade #desenvolvimentopessoal</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2025-09-12 20:59:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>corte_3_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>batman-e-a-luta-interna.mp4</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Batman e a luta interna</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Como lembrar de quem você é para enfrentar desafios. @desenvolvimentopessoal #identidade #autopercepção</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>#batman #lutainternar #autopercepção</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>60.01</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2025-09-12 20:59:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>corte_4_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>lembrar-quem-voce-e.mp4</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Lembrar quem você é</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Veja como a memória de identidade pode te libertar. Batman perdeu a lembrança do seu verdadeiro eu e ficou preso em um trabalho forçado até que recordou quem era realmente. #memoriaidentidade #desenvolvimentopessoal</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>#memoriaidentidade #desenvolvimentopessoal #identidadedepessoas</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>25.02</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2025-09-12 20:59:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>corte_5_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>influencia-vs-controle.mp4</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Influência vs Controle</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Entenda a diferença entre influenciar e tentar controlar coisas fora do seu alcance. Foco no 'jogo interno' traz vitória duradoura. #autoconhecimento #desenvolvimentopessoal</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>#influenciavcontrolo #autodeterminacao #vitorguerreireal</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>59.01</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2025-09-12 20:59:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>corte_6_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>aprendendo-a-valorizar-o-presente.mp4</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Aprendendo a valorizar o presente</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Entenda como apreciar o que temos agora pode nos ajudar a olhar para o futuro com esperança. #aprendizado #atitudepositiva</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>#aprendizado #atitudepositiva #futuromelhor</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>35.03</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2025-09-12 21:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>corte_1_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>como-superar-a-ansiedade-matinal.mp4</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Como superar a ansiedade matinal</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Acordando com ansiedade? Descubra como transformar este medo diário em motivação para o sucesso. Papai e mamãe não vão mais te acordar, você fará isso sozinho! 🌟 #motivação #ansiedade #sucesso</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>#motivação #ansiedade #sucesso</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>54</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2025-09-13 18:04:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>corte_2_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>conversas-sozinho-sao-essenciais.mp4</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Conversas sozinho são essenciais</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Spending time alone allows growth. Conversar consigo mesmo é crucial para o desenvolvimento pessoal. Vamos valorizar momentos de introspecção.</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>#desenvolvimentopessoal #solitude #conversassozinho</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>57.01</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2025-09-13 18:04:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>corte_3_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>passar-tempo-sozinho-para-se-destacar.mp4</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Passar tempo sozinho para se destacar</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Pessoas de sucesso têm a habilidade de passar tempo sozinho, entendendo seus comportamentos e crenças. Desenvolva essa superpotência para ficar à frente da concorrência! 🚀💪 #sucesso #superpotencia #tempoversoziho</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>#sucesso #superpotencia #tempoversoziho</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>55</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2025-09-13 18:04:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>corte_1_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>padroes-e-sucesso-no-marketing-digital.mp4</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Padrões e Sucesso no Marketing Digital</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Entenda como reconhecer e usar padrões para o seu sucesso no marketing digital. Veja o caso da Amazon e Tom Brady! #padroes #sucesso #marketingdigital</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>#padroes #sucesso #marketingdigital</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>40.03</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>2025-09-21 11:32:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>corte_4_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>auto-estima-e-sucesso-pessoal.mp4</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Auto-estima e sucesso pessoal</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Você tem controle sobre sua auto-estima. Descubra quem você é ao fazer coisas difíceis! Não se deixe influenciar por o que os outros dizem.</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>#autoestima #sucesso #conquista</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>25.02</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>2025-09-21 11:33:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>corte_6_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>aprendendo-a-apreciar-o-momento.mp4</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Aprendendo a apreciar o momento</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Se tudo muda e termina, aprenda a valorizar o que tem agora. E trabalhe para tornar o futuro melhor! #aprendizagem #autoaperfeiçoamento #motivação</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>#aprendizagem #autoaperfeiçoamento #motivação</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>35.03</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>2025-09-21 11:33:14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
✅ DUBLAGEM PERFEITA - XTTS v2 com sincronização e clonagem de voz
🎯 CORREÇÕES IMPLEMENTADAS:
- ✅ Corrigido time-stretching com atempo (preserva timbre natural)
- ✅ Inversão correta do ratio para atempo (elimina câmera lenta)
- ✅ Sincronização perfeita com legendas
- ✅ Clonagem de voz natural (sem efeito Minion/Darth Vader)
- ✅ GPU + CPU otimizado (comportamento normal e eficiente)
- ✅ Limites inteligentes de aceleração (máximo 2.5x)
- ✅ Fallback CPU robusto para PyTorch 2.6

🎤 RESULTADO:
- Voz natural e sincronizada
- Qualidade de clonagem perfeita
- Performance otimizada
- Sistema estável e confiável
</commit_message>
<xml_diff>
--- a/metadados/videos.xlsx
+++ b/metadados/videos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4388,6 +4388,76 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>corte_1_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>motivacao-familiar-na-rotina.mp4</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Motivação familiar na rotina</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Você sente falta de motivar-se? Pense em mama e o dia do draft. Motivação vem da família! 🤝 #motivaçãofamiliar #diasdifíceis #famíliaéchave</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>#motivaçãofamiliar #diasdifíceis #famíliaéchave</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>36.03</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>2025-09-22 10:25:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>corte_4_legendado.mp4</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>motivacao-matinal-para-instagram.mp4</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Motivação matinal para Instagram</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Eu acordo às 3 da manhã e posto vídeos no Instagram porque quero ser o melhor. Honorando Dr. King e Malcolm X, assim como os atletas do Hall of Fame! #motivação #instagram #manhãacordada</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>#motivação #instagram #manhãacordada</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>21.02</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>2025-09-22 10:26:06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>